<commit_message>
Git sh to ease commit and push
</commit_message>
<xml_diff>
--- a/controlRoom_server/server/templates/ICR_TEMPLATE018.xlsx
+++ b/controlRoom_server/server/templates/ICR_TEMPLATE018.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10703"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C8DDC89-7567-0647-B791-E73648F27834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C05B6EFF-762D-644B-AD76-023109DBCFC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3740" yWindow="340" windowWidth="20440" windowHeight="16460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="640" windowWidth="20440" windowHeight="16460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ICR_TEMPLATE018.xlsx" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>SITE_CODE</t>
   </si>
@@ -42,22 +42,22 @@
     <t>QTY</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>0</t>
   </si>
   <si>
-    <t>90061</t>
-  </si>
-  <si>
-    <t>189599</t>
-  </si>
-  <si>
-    <t>60.72</t>
-  </si>
-  <si>
-    <t>CASE_COST</t>
+    <t>UNIT_COST</t>
+  </si>
+  <si>
+    <t>POSITION</t>
+  </si>
+  <si>
+    <t>ALL</t>
+  </si>
+  <si>
+    <t>301229</t>
+  </si>
+  <si>
+    <t>5.24</t>
   </si>
 </sst>
 </file>
@@ -67,9 +67,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -145,23 +152,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -477,20 +487,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="16.1640625" style="3" customWidth="1"/>
-    <col min="4" max="5" width="13" style="3" customWidth="1"/>
-    <col min="6" max="10" width="10.83203125" style="3" customWidth="1"/>
-    <col min="11" max="11" width="65" style="3" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" style="3" customWidth="1"/>
-    <col min="13" max="16384" width="10.83203125" style="3"/>
+    <col min="3" max="4" width="16.1640625" style="3" customWidth="1"/>
+    <col min="5" max="6" width="13" style="3" customWidth="1"/>
+    <col min="7" max="11" width="10.83203125" style="3" customWidth="1"/>
+    <col min="12" max="12" width="65" style="3" customWidth="1"/>
+    <col min="13" max="13" width="10.83203125" style="3" customWidth="1"/>
+    <col min="14" max="16384" width="10.83203125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -501,27 +511,33 @@
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>9</v>
+      <c r="F1" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="5" t="s">
+    <row r="2" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
         <v>7</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>5</v>
+      <c r="D2" s="6" t="s">
+        <v>7</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>